<commit_message>
fix(productos): Fase A — 18 kits de tareas v1.1 (todos menos pastelería, ya v2.0): Nº de tarea en col. A, columna «✓ Completada» con desplegable ✓/—/N/A, fila verde al marcar, contador con numerador y denominador calculados (o desplegable en la columna OK en los kits de origen CB), cache de valores, A4, metadata, bio anclada, versión
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016924EP7QJuq6BNFj8S7Fks
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/kit-tareas-asador/01-apertura-cierre-asador.xlsx
+++ b/astro-site/public/dl/kit-tareas-asador/01-apertura-cierre-asador.xlsx
@@ -11,7 +11,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Apertura Parrilla y Josper" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cierre Parrilla y Josper" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Apertura Parrilla y Josper'!$4:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Cierre Parrilla y Josper'!$4:$4</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -19,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -64,6 +67,16 @@
       <color rgb="00999999"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00666666"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -100,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -120,10 +133,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00C8E6C9"/>
+          <bgColor rgb="00C8E6C9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -484,14 +511,15 @@
   <sheetPr>
     <tabColor rgb="00C4974A"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:B19"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -499,6 +527,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="B4" s="2" t="inlineStr">
         <is>
@@ -506,6 +535,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="B6" s="3" t="inlineStr">
         <is>
@@ -541,6 +571,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="B12" s="2" t="inlineStr">
         <is>
@@ -548,6 +579,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="B14" s="3" t="inlineStr">
         <is>
@@ -576,6 +608,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="B19" s="2" t="inlineStr">
         <is>
@@ -583,8 +616,33 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
+    <row r="21">
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Marca con ✓ en la columna «✓ Completada» (desplegable): es la que cuenta el total de tareas completadas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Versión 1.1 · agosto 2026 · aichef.pro/kit-tareas-asador · info@aichef.pro</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;8 AI Chef Pro · aichef.pro · Página &amp;P de &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -593,7 +651,7 @@
   <sheetPr>
     <tabColor rgb="008B4513"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -621,10 +679,11 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>Nº</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
@@ -649,7 +708,7 @@
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>Hecha</t>
+          <t>✓ Completada</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -666,10 +725,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A6" s="13" t="n">
+        <v>1</v>
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
@@ -695,10 +752,8 @@
       <c r="G6" s="10" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A7" s="13" t="n">
+        <v>2</v>
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
@@ -724,10 +779,8 @@
       <c r="G7" s="10" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A8" s="13" t="n">
+        <v>3</v>
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
@@ -753,10 +806,8 @@
       <c r="G8" s="10" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A9" s="13" t="n">
+        <v>4</v>
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
@@ -782,10 +833,8 @@
       <c r="G9" s="10" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A10" s="13" t="n">
+        <v>5</v>
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
@@ -811,10 +860,8 @@
       <c r="G10" s="10" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A11" s="13" t="n">
+        <v>6</v>
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
@@ -840,10 +887,8 @@
       <c r="G11" s="10" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A12" s="13" t="n">
+        <v>7</v>
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
@@ -869,10 +914,8 @@
       <c r="G12" s="10" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A13" s="13" t="n">
+        <v>8</v>
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
@@ -898,10 +941,8 @@
       <c r="G13" s="10" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A14" s="13" t="n">
+        <v>9</v>
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
@@ -926,6 +967,7 @@
       <c r="F14" s="9" t="n"/>
       <c r="G14" s="10" t="n"/>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
@@ -934,10 +976,8 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A17" s="13" t="n">
+        <v>10</v>
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
@@ -963,10 +1003,8 @@
       <c r="G17" s="10" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A18" s="13" t="n">
+        <v>11</v>
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
@@ -992,10 +1030,8 @@
       <c r="G18" s="10" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A19" s="13" t="n">
+        <v>12</v>
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
@@ -1021,10 +1057,8 @@
       <c r="G19" s="10" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A20" s="13" t="n">
+        <v>13</v>
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
@@ -1050,10 +1084,8 @@
       <c r="G20" s="10" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A21" s="13" t="n">
+        <v>14</v>
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
@@ -1078,6 +1110,7 @@
       <c r="F21" s="9" t="n"/>
       <c r="G21" s="10" t="n"/>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
@@ -1086,10 +1119,8 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A24" s="13" t="n">
+        <v>15</v>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
@@ -1115,10 +1146,8 @@
       <c r="G24" s="10" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A25" s="13" t="n">
+        <v>16</v>
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
@@ -1144,10 +1173,8 @@
       <c r="G25" s="10" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A26" s="13" t="n">
+        <v>17</v>
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
@@ -1173,10 +1200,8 @@
       <c r="G26" s="10" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A27" s="13" t="n">
+        <v>18</v>
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
@@ -1202,10 +1227,8 @@
       <c r="G27" s="10" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A28" s="13" t="n">
+        <v>19</v>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
@@ -1231,10 +1254,8 @@
       <c r="G28" s="10" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A29" s="13" t="n">
+        <v>20</v>
       </c>
       <c r="B29" s="10" t="inlineStr">
         <is>
@@ -1259,6 +1280,7 @@
       <c r="F29" s="9" t="n"/>
       <c r="G29" s="10" t="n"/>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
@@ -1267,10 +1289,8 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A32" s="13" t="n">
+        <v>21</v>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
@@ -1296,10 +1316,8 @@
       <c r="G32" s="10" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A33" s="13" t="n">
+        <v>22</v>
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
@@ -1325,10 +1343,8 @@
       <c r="G33" s="10" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A34" s="13" t="n">
+        <v>23</v>
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
@@ -1354,10 +1370,8 @@
       <c r="G34" s="10" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A35" s="13" t="n">
+        <v>24</v>
       </c>
       <c r="B35" s="10" t="inlineStr">
         <is>
@@ -1381,6 +1395,27 @@
       </c>
       <c r="F35" s="9" t="n"/>
       <c r="G35" s="10" t="n"/>
+    </row>
+    <row r="36"/>
+    <row r="37">
+      <c r="A37" s="14" t="inlineStr">
+        <is>
+          <t>Tareas completadas:</t>
+        </is>
+      </c>
+      <c r="D37">
+        <f>COUNTIF(F5:F35,"✓")</f>
+        <v>0.0</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="F37">
+        <f>COUNTIF(B5:B35,"?*")</f>
+        <v>24.0</v>
+      </c>
     </row>
     <row r="38">
       <c r="B38" s="12" t="inlineStr">
@@ -1402,10 +1437,29 @@
     <mergeCell ref="A31:G31"/>
     <mergeCell ref="A16:G16"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A23:G23"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A23:G23"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <conditionalFormatting sqref="A5:G35">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>$F5="✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="F6 F7 F8 F9 F10 F11 F12 F13 F14 F17 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F32 F33 F34 F35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"✓,—,N/A"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;8 AI Chef Pro · aichef.pro · Página &amp;P de &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -1414,7 +1468,7 @@
   <sheetPr>
     <tabColor rgb="00C4974A"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1442,10 +1496,11 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>Nº</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
@@ -1470,7 +1525,7 @@
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>Hecha</t>
+          <t>✓ Completada</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -1487,10 +1542,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A6" s="13" t="n">
+        <v>1</v>
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
@@ -1516,10 +1569,8 @@
       <c r="G6" s="10" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A7" s="13" t="n">
+        <v>2</v>
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
@@ -1545,10 +1596,8 @@
       <c r="G7" s="10" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A8" s="13" t="n">
+        <v>3</v>
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
@@ -1574,10 +1623,8 @@
       <c r="G8" s="10" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A9" s="13" t="n">
+        <v>4</v>
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
@@ -1603,10 +1650,8 @@
       <c r="G9" s="10" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A10" s="13" t="n">
+        <v>5</v>
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
@@ -1631,6 +1676,7 @@
       <c r="F10" s="9" t="n"/>
       <c r="G10" s="10" t="n"/>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
@@ -1639,10 +1685,8 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A13" s="13" t="n">
+        <v>6</v>
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
@@ -1668,10 +1712,8 @@
       <c r="G13" s="10" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A14" s="13" t="n">
+        <v>7</v>
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
@@ -1697,10 +1739,8 @@
       <c r="G14" s="10" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A15" s="13" t="n">
+        <v>8</v>
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
@@ -1726,10 +1766,8 @@
       <c r="G15" s="10" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A16" s="13" t="n">
+        <v>9</v>
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
@@ -1755,10 +1793,8 @@
       <c r="G16" s="10" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A17" s="13" t="n">
+        <v>10</v>
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
@@ -1783,6 +1819,7 @@
       <c r="F17" s="9" t="n"/>
       <c r="G17" s="10" t="n"/>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
@@ -1791,10 +1828,8 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A20" s="13" t="n">
+        <v>11</v>
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
@@ -1820,10 +1855,8 @@
       <c r="G20" s="10" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A21" s="13" t="n">
+        <v>12</v>
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
@@ -1849,10 +1882,8 @@
       <c r="G21" s="10" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A22" s="13" t="n">
+        <v>13</v>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
@@ -1878,10 +1909,8 @@
       <c r="G22" s="10" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A23" s="13" t="n">
+        <v>14</v>
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
@@ -1907,10 +1936,8 @@
       <c r="G23" s="10" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A24" s="13" t="n">
+        <v>15</v>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
@@ -1936,10 +1963,8 @@
       <c r="G24" s="10" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A25" s="13" t="n">
+        <v>16</v>
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
@@ -1965,10 +1990,8 @@
       <c r="G25" s="10" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A26" s="13" t="n">
+        <v>17</v>
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
@@ -1994,10 +2017,8 @@
       <c r="G26" s="10" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="9" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
+      <c r="A27" s="13" t="n">
+        <v>18</v>
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
@@ -2022,6 +2043,27 @@
       <c r="F27" s="9" t="n"/>
       <c r="G27" s="10" t="n"/>
     </row>
+    <row r="28"/>
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr">
+        <is>
+          <t>Tareas completadas:</t>
+        </is>
+      </c>
+      <c r="D29">
+        <f>COUNTIF(F5:F27,"✓")</f>
+        <v>0.0</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="F29">
+        <f>COUNTIF(B5:B27,"?*")</f>
+        <v>18.0</v>
+      </c>
+    </row>
     <row r="30">
       <c r="B30" s="12" t="inlineStr">
         <is>
@@ -2038,12 +2080,31 @@
     </row>
   </sheetData>
   <mergeCells count="5">
+    <mergeCell ref="A12:G12"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A12:G12"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A19:G19"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <conditionalFormatting sqref="A5:G27">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>$F5="✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="F6 F7 F8 F9 F10 F13 F14 F15 F16 F17 F20 F21 F22 F23 F24 F25 F26 F27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"✓,—,N/A"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;8 AI Chef Pro · aichef.pro · Página &amp;P de &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>